<commit_message>
docs: reconstruir seguimiento de riesgos como matriz semanal de trayectoria (nivel por semana + resumen)
</commit_message>
<xml_diff>
--- a/docs/Plan_Riesgos.xlsx
+++ b/docs/Plan_Riesgos.xlsx
@@ -9,7 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riesgos_actuales" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora_seguimiento" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Riesgo_Servicio" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento_semanal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz_Riesgo_Servicio" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +86,54 @@
       <color rgb="FFC00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -142,8 +190,38 @@
         <fgColor rgb="FFFAFAFA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E06666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0093C47D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -199,11 +277,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -300,6 +392,62 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -686,11 +834,10 @@
     <row r="2" ht="36" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Riesgos del proyecto con su evaluación, plan de mitigación y bitácora de seguimiento. Documento vivo: se actualiza cada sprint planning conforme los riesgos evolucionan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Riesgos del proyecto con su evaluación, plan de mitigación y bitácora de seguimiento. Documento vivo: se actualiza semanalmente en el reporte de seguimiento (hoja Reporte_semanal) conforme los riesgos evolucionan.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="21.95" customHeight="1" s="32">
       <c r="A4" s="29" t="inlineStr">
         <is>
@@ -735,7 +882,6 @@
       </c>
       <c r="H5" s="30" t="n"/>
     </row>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="32">
       <c r="A7" s="31" t="inlineStr">
         <is>
@@ -885,8 +1031,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16" ht="15.75" customHeight="1" s="32">
       <c r="A16" s="31" t="inlineStr">
         <is>
@@ -1489,11 +1633,10 @@
     <row r="2" ht="30" customHeight="1" s="32">
       <c r="A2" s="33" t="inlineStr">
         <is>
-          <t>Detalle completo de cada riesgo. Esta tabla se actualiza cada sprint planning. Los cambios de estado se registran en la hoja Bitácora_seguimiento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Detalle completo de cada riesgo. Esta tabla se actualiza semanalmente en el reporte de seguimiento (hoja Reporte_semanal). Cada sprint dura una semana. Los cambios de estado se registran en la hoja Bitácora_seguimiento.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="30" customHeight="1" s="32">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -2145,7 +2288,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="32.1" customHeight="1" s="32">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -2768,6 +2910,1631 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AB15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" style="32" min="1" max="1"/>
+    <col width="16" customWidth="1" style="32" min="2" max="2"/>
+    <col width="30" customWidth="1" style="32" min="3" max="3"/>
+    <col width="40" customWidth="1" style="32" min="4" max="4"/>
+    <col width="10" customWidth="1" style="32" min="5" max="5"/>
+    <col width="9" customWidth="1" style="32" min="6" max="6"/>
+    <col width="11" customWidth="1" style="32" min="7" max="7"/>
+    <col width="38" customWidth="1" style="32" min="8" max="8"/>
+    <col width="9" customWidth="1" style="32" min="9" max="9"/>
+    <col width="9" customWidth="1" style="32" min="10" max="10"/>
+    <col width="9" customWidth="1" style="32" min="11" max="11"/>
+    <col width="9" customWidth="1" style="32" min="12" max="12"/>
+    <col width="9" customWidth="1" style="32" min="13" max="13"/>
+    <col width="9" customWidth="1" style="32" min="14" max="14"/>
+    <col width="9" customWidth="1" style="32" min="15" max="15"/>
+    <col width="9" customWidth="1" style="32" min="16" max="16"/>
+    <col width="9" customWidth="1" style="32" min="17" max="17"/>
+    <col width="9" customWidth="1" style="32" min="18" max="18"/>
+    <col width="9" customWidth="1" style="32" min="19" max="19"/>
+    <col width="9" customWidth="1" style="32" min="20" max="20"/>
+    <col width="9" customWidth="1" style="32" min="21" max="21"/>
+    <col width="9" customWidth="1" style="32" min="22" max="22"/>
+    <col width="9" customWidth="1" style="32" min="23" max="23"/>
+    <col width="9" customWidth="1" style="32" min="24" max="24"/>
+    <col width="9" customWidth="1" style="32" min="25" max="25"/>
+    <col width="9" customWidth="1" style="32" min="26" max="26"/>
+    <col width="9" customWidth="1" style="32" min="27" max="27"/>
+    <col width="9" customWidth="1" style="32" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="inlineStr">
+        <is>
+          <t>Seguimiento semanal de riesgos — SIGECOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="46" t="inlineStr">
+        <is>
+          <t>Escala cualitativa del nivel de riesgo: ALTA · MEDIA · BAJA · NULA. Cada columna es una semana (un sprint). Celda vacía = semana sin seguimiento registrado. El seguimiento formal inició el 10/05/2026 (S14). Proyecto: 03/02–15/06/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="32">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Riesgo_ID</t>
+        </is>
+      </c>
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C3" s="47" t="inlineStr">
+        <is>
+          <t>Riesgo</t>
+        </is>
+      </c>
+      <c r="D3" s="47" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="E3" s="47" t="inlineStr">
+        <is>
+          <t>Prob. inicial</t>
+        </is>
+      </c>
+      <c r="F3" s="47" t="inlineStr">
+        <is>
+          <t>Impacto</t>
+        </is>
+      </c>
+      <c r="G3" s="47" t="inlineStr">
+        <is>
+          <t>Nivel inicial</t>
+        </is>
+      </c>
+      <c r="H3" s="47" t="inlineStr">
+        <is>
+          <t>Mitigación</t>
+        </is>
+      </c>
+      <c r="I3" s="47" t="inlineStr">
+        <is>
+          <t>S1
+02/02–08/02</t>
+        </is>
+      </c>
+      <c r="J3" s="47" t="inlineStr">
+        <is>
+          <t>S2
+09/02–15/02</t>
+        </is>
+      </c>
+      <c r="K3" s="47" t="inlineStr">
+        <is>
+          <t>S3
+16/02–22/02</t>
+        </is>
+      </c>
+      <c r="L3" s="47" t="inlineStr">
+        <is>
+          <t>S4
+23/02–01/03</t>
+        </is>
+      </c>
+      <c r="M3" s="47" t="inlineStr">
+        <is>
+          <t>S5
+02/03–08/03</t>
+        </is>
+      </c>
+      <c r="N3" s="47" t="inlineStr">
+        <is>
+          <t>S6
+09/03–15/03</t>
+        </is>
+      </c>
+      <c r="O3" s="47" t="inlineStr">
+        <is>
+          <t>S7
+16/03–22/03</t>
+        </is>
+      </c>
+      <c r="P3" s="47" t="inlineStr">
+        <is>
+          <t>S8
+23/03–29/03</t>
+        </is>
+      </c>
+      <c r="Q3" s="47" t="inlineStr">
+        <is>
+          <t>S9
+30/03–05/04</t>
+        </is>
+      </c>
+      <c r="R3" s="47" t="inlineStr">
+        <is>
+          <t>S10
+06/04–12/04</t>
+        </is>
+      </c>
+      <c r="S3" s="47" t="inlineStr">
+        <is>
+          <t>S11
+13/04–19/04</t>
+        </is>
+      </c>
+      <c r="T3" s="47" t="inlineStr">
+        <is>
+          <t>S12
+20/04–26/04</t>
+        </is>
+      </c>
+      <c r="U3" s="47" t="inlineStr">
+        <is>
+          <t>S13
+27/04–03/05</t>
+        </is>
+      </c>
+      <c r="V3" s="47" t="inlineStr">
+        <is>
+          <t>S14
+04/05–10/05</t>
+        </is>
+      </c>
+      <c r="W3" s="47" t="inlineStr">
+        <is>
+          <t>S15
+11/05–17/05</t>
+        </is>
+      </c>
+      <c r="X3" s="47" t="inlineStr">
+        <is>
+          <t>S16
+18/05–24/05</t>
+        </is>
+      </c>
+      <c r="Y3" s="47" t="inlineStr">
+        <is>
+          <t>S17
+25/05–31/05</t>
+        </is>
+      </c>
+      <c r="Z3" s="47" t="inlineStr">
+        <is>
+          <t>S18
+01/06–07/06</t>
+        </is>
+      </c>
+      <c r="AA3" s="47" t="inlineStr">
+        <is>
+          <t>S19
+08/06–14/06</t>
+        </is>
+      </c>
+      <c r="AB3" s="47" t="inlineStr">
+        <is>
+          <t>S20
+15/06–21/06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1" s="32">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>R-01</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>Curva de aprendizaje de React excede el primer sprint</t>
+        </is>
+      </c>
+      <c r="D4" s="49" t="inlineStr">
+        <is>
+          <t>El equipo no tiene experiencia previa con React. Si el aprendizaje se hace en paralelo al Sprint 1, las historias HU-00, HU-01 y HU-08 pueden no quedar terminadas a tiempo, atrasando el resto del cronograma.</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F4" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
+        <is>
+          <t>Reservar la semana anterior al Sprint 1 para tutoriales oficiales de React + Tailwind. Construir una plantilla base con login y rutas configuradas antes de tocar las historias. Usar componentes pre-hechos de shadcn/ui en lugar de construir todo desde cero.</t>
+        </is>
+      </c>
+      <c r="I4" s="50" t="n"/>
+      <c r="J4" s="50" t="n"/>
+      <c r="K4" s="50" t="n"/>
+      <c r="L4" s="50" t="n"/>
+      <c r="M4" s="50" t="n"/>
+      <c r="N4" s="50" t="n"/>
+      <c r="O4" s="50" t="n"/>
+      <c r="P4" s="50" t="n"/>
+      <c r="Q4" s="50" t="n"/>
+      <c r="R4" s="50" t="n"/>
+      <c r="S4" s="50" t="n"/>
+      <c r="T4" s="50" t="n"/>
+      <c r="U4" s="50" t="n"/>
+      <c r="V4" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="W4" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X4" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y4" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z4" s="50" t="n"/>
+      <c r="AA4" s="50" t="n"/>
+      <c r="AB4" s="50" t="n"/>
+    </row>
+    <row r="5" ht="46" customHeight="1" s="32">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>R-02</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>Configuración de Docker en local consume tiempo del Sprint 1</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>Instalar Docker en las tres laptops del equipo y configurar el docker-compose con Node, PostgreSQL y volúmenes correctamente puede consumir 1-2 días si surge cualquier incompatibilidad con Windows, Mac o el firewall.</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F5" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H5" s="49" t="inlineStr">
+        <is>
+          <t>Preparar un Dockerfile y docker-compose.yml validado antes del Sprint 1. Documentar los pasos exactos de instalación para los tres integrantes. Hacer una sesión grupal de instalación inicial donde todos resuelvan dudas juntos.</t>
+        </is>
+      </c>
+      <c r="I5" s="50" t="n"/>
+      <c r="J5" s="50" t="n"/>
+      <c r="K5" s="50" t="n"/>
+      <c r="L5" s="50" t="n"/>
+      <c r="M5" s="50" t="n"/>
+      <c r="N5" s="50" t="n"/>
+      <c r="O5" s="50" t="n"/>
+      <c r="P5" s="50" t="n"/>
+      <c r="Q5" s="50" t="n"/>
+      <c r="R5" s="50" t="n"/>
+      <c r="S5" s="50" t="n"/>
+      <c r="T5" s="50" t="n"/>
+      <c r="U5" s="50" t="n"/>
+      <c r="V5" s="50" t="n"/>
+      <c r="W5" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="X5" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Y5" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Z5" s="50" t="n"/>
+      <c r="AA5" s="50" t="n"/>
+      <c r="AB5" s="50" t="n"/>
+    </row>
+    <row r="6" ht="46" customHeight="1" s="32">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>R-03</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>Diseño de base de datos inicial incompleto requiere migraciones tardías</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>Si el modelo de datos se diseña sobre la marcha, los Sprints 3-5 requerirán migraciones frecuentes que pueden romper datos de pruebas y consumir tiempo de desarrollo.</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F6" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H6" s="49" t="inlineStr">
+        <is>
+          <t>Diseñar el modelo de datos completo en la primera semana, con revisión cruzada del equipo. Usar Prisma o Knex como herramienta de migración para gestionar cambios al esquema sin pérdida de datos.</t>
+        </is>
+      </c>
+      <c r="I6" s="50" t="n"/>
+      <c r="J6" s="50" t="n"/>
+      <c r="K6" s="50" t="n"/>
+      <c r="L6" s="50" t="n"/>
+      <c r="M6" s="50" t="n"/>
+      <c r="N6" s="50" t="n"/>
+      <c r="O6" s="50" t="n"/>
+      <c r="P6" s="50" t="n"/>
+      <c r="Q6" s="50" t="n"/>
+      <c r="R6" s="50" t="n"/>
+      <c r="S6" s="50" t="n"/>
+      <c r="T6" s="50" t="n"/>
+      <c r="U6" s="50" t="n"/>
+      <c r="V6" s="50" t="n"/>
+      <c r="W6" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="X6" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Y6" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Z6" s="50" t="n"/>
+      <c r="AA6" s="50" t="n"/>
+      <c r="AB6" s="50" t="n"/>
+    </row>
+    <row r="7" ht="46" customHeight="1" s="32">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>R-04</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>Despliegue inicial en Render falla por configuración</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>El primer despliegue suele tener problemas de configuración: variables de entorno, puertos, conexión a la base de datos PostgreSQL de Render, certificados SSL.</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F7" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H7" s="49" t="inlineStr">
+        <is>
+          <t>Realizar el primer despliegue al final del Sprint 1 con la versión mínima del sistema. Identificar y resolver problemas temprano, no en el sprint final.</t>
+        </is>
+      </c>
+      <c r="I7" s="50" t="n"/>
+      <c r="J7" s="50" t="n"/>
+      <c r="K7" s="50" t="n"/>
+      <c r="L7" s="50" t="n"/>
+      <c r="M7" s="50" t="n"/>
+      <c r="N7" s="50" t="n"/>
+      <c r="O7" s="50" t="n"/>
+      <c r="P7" s="50" t="n"/>
+      <c r="Q7" s="50" t="n"/>
+      <c r="R7" s="50" t="n"/>
+      <c r="S7" s="50" t="n"/>
+      <c r="T7" s="50" t="n"/>
+      <c r="U7" s="50" t="n"/>
+      <c r="V7" s="50" t="n"/>
+      <c r="W7" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X7" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y7" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z7" s="50" t="n"/>
+      <c r="AA7" s="50" t="n"/>
+      <c r="AB7" s="50" t="n"/>
+    </row>
+    <row r="8" ht="46" customHeight="1" s="32">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>R-05</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>Técnico</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>Render aplica suspensión por inactividad en el plan gratuito</t>
+        </is>
+      </c>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>El plan gratuito de Render suspende los servicios sin uso durante 15 minutos. Al volver a accederlos toma 30-60 segundos en arrancar, lo que puede dar mala impresión en la demo.</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F8" s="48" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G8" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H8" s="49" t="inlineStr">
+        <is>
+          <t>Documentar al cliente que este comportamiento corresponde al plan gratuito y no al sistema. Antes de cada demo, abrir la URL 5 minutos antes para mantener el servicio activo. Considerar upgrade al plan pagado solo si es crítico.</t>
+        </is>
+      </c>
+      <c r="I8" s="50" t="n"/>
+      <c r="J8" s="50" t="n"/>
+      <c r="K8" s="50" t="n"/>
+      <c r="L8" s="50" t="n"/>
+      <c r="M8" s="50" t="n"/>
+      <c r="N8" s="50" t="n"/>
+      <c r="O8" s="50" t="n"/>
+      <c r="P8" s="50" t="n"/>
+      <c r="Q8" s="50" t="n"/>
+      <c r="R8" s="50" t="n"/>
+      <c r="S8" s="50" t="n"/>
+      <c r="T8" s="50" t="n"/>
+      <c r="U8" s="50" t="n"/>
+      <c r="V8" s="50" t="n"/>
+      <c r="W8" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X8" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y8" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z8" s="50" t="n"/>
+      <c r="AA8" s="50" t="n"/>
+      <c r="AB8" s="50" t="n"/>
+    </row>
+    <row r="9" ht="46" customHeight="1" s="32">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="inlineStr">
+        <is>
+          <t>Velocidad real del equipo es menor a 9 puntos por sprint</t>
+        </is>
+      </c>
+      <c r="D9" s="49" t="inlineStr">
+        <is>
+          <t>El plan iterativo asume 9 puntos por sprint (3 personas × 3 días útiles × 1 punto por día-persona), velocidad consolidada con el cliente en la revisión del 18/05/2026. Si el equipo solo logra 5-7 puntos reales, el cronograma de 9 semanas falla y hay que recortar alcance o renegociar entregas al cierre del Sprint 1, una vez medida la velocidad real.</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F9" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G9" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H9" s="49" t="inlineStr">
+        <is>
+          <t>Tras el Sprint 1, recalibrar la velocidad real del equipo. Si es menor a lo estimado, ajustar puntos de las historias siguientes o priorizar Etapa 1 sobre funcionalidades opcionales. No insistir con el estimado original si la realidad lo desmiente.</t>
+        </is>
+      </c>
+      <c r="I9" s="50" t="n"/>
+      <c r="J9" s="50" t="n"/>
+      <c r="K9" s="50" t="n"/>
+      <c r="L9" s="50" t="n"/>
+      <c r="M9" s="50" t="n"/>
+      <c r="N9" s="50" t="n"/>
+      <c r="O9" s="50" t="n"/>
+      <c r="P9" s="50" t="n"/>
+      <c r="Q9" s="50" t="n"/>
+      <c r="R9" s="50" t="n"/>
+      <c r="S9" s="50" t="n"/>
+      <c r="T9" s="50" t="n"/>
+      <c r="U9" s="50" t="n"/>
+      <c r="V9" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="W9" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="X9" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y9" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z9" s="50" t="n"/>
+      <c r="AA9" s="50" t="n"/>
+      <c r="AB9" s="50" t="n"/>
+    </row>
+    <row r="10" ht="46" customHeight="1" s="32">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>R-07</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>Conflictos de merge frecuentes por trabajo paralelo</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>Tres integrantes trabajando simultáneamente en el mismo repositorio pueden generar conflictos de merge en archivos compartidos (estilos, rutas, configuraciones), consumiendo tiempo de desarrollo.</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H10" s="49" t="inlineStr">
+        <is>
+          <t>Establecer convenciones de ramas: una rama por historia (feature/HU-XX), commits frecuentes, revisión por pull request antes de hacer merge a main. Reuniones diarias de 10 minutos para detectar conflictos antes de que crezcan.</t>
+        </is>
+      </c>
+      <c r="I10" s="50" t="n"/>
+      <c r="J10" s="50" t="n"/>
+      <c r="K10" s="50" t="n"/>
+      <c r="L10" s="50" t="n"/>
+      <c r="M10" s="50" t="n"/>
+      <c r="N10" s="50" t="n"/>
+      <c r="O10" s="50" t="n"/>
+      <c r="P10" s="50" t="n"/>
+      <c r="Q10" s="50" t="n"/>
+      <c r="R10" s="50" t="n"/>
+      <c r="S10" s="50" t="n"/>
+      <c r="T10" s="50" t="n"/>
+      <c r="U10" s="50" t="n"/>
+      <c r="V10" s="50" t="n"/>
+      <c r="W10" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X10" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y10" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z10" s="50" t="n"/>
+      <c r="AA10" s="50" t="n"/>
+      <c r="AB10" s="50" t="n"/>
+    </row>
+    <row r="11" ht="46" customHeight="1" s="32">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>R-08</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="inlineStr">
+        <is>
+          <t>Ausencia temporal de un integrante por carga académica o salud</t>
+        </is>
+      </c>
+      <c r="D11" s="49" t="inlineStr">
+        <is>
+          <t>El equipo de 3 personas no tiene margen para perder integrantes durante semanas críticas. Una ausencia de 1 semana en sprint pico puede atrasar el proyecto.</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F11" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G11" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H11" s="49" t="inlineStr">
+        <is>
+          <t>Documentar cada historia entregada para que cualquier integrante pueda retomar el código de otro. Sincronización en GitHub al final de cada día. Tener un sprint de holgura al final del cronograma como buffer.</t>
+        </is>
+      </c>
+      <c r="I11" s="50" t="n"/>
+      <c r="J11" s="50" t="n"/>
+      <c r="K11" s="50" t="n"/>
+      <c r="L11" s="50" t="n"/>
+      <c r="M11" s="50" t="n"/>
+      <c r="N11" s="50" t="n"/>
+      <c r="O11" s="50" t="n"/>
+      <c r="P11" s="50" t="n"/>
+      <c r="Q11" s="50" t="n"/>
+      <c r="R11" s="50" t="n"/>
+      <c r="S11" s="50" t="n"/>
+      <c r="T11" s="50" t="n"/>
+      <c r="U11" s="50" t="n"/>
+      <c r="V11" s="50" t="n"/>
+      <c r="W11" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="X11" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Y11" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Z11" s="50" t="n"/>
+      <c r="AA11" s="50" t="n"/>
+      <c r="AB11" s="50" t="n"/>
+    </row>
+    <row r="12" ht="46" customHeight="1" s="32">
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>R-09</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>El cliente solicita cambios mayores de alcance que rompen historias ya implementadas</t>
+        </is>
+      </c>
+      <c r="D12" s="49" t="inlineStr">
+        <is>
+          <t>Como ocurrió con el cambio del módulo 7 y la fusión de servicios, el cliente puede solicitar cambios estructurales en revisiones futuras que obligan a rehacer trabajo ya completado.</t>
+        </is>
+      </c>
+      <c r="E12" s="48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F12" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G12" s="48" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="H12" s="49" t="inlineStr">
+        <is>
+          <t>Presentar maquetas y prototipos ANTES de programar para obtener aprobación temprana. Cualquier cambio mayor solicitado después del Sprint 2 requiere ajuste explícito del cronograma. Documentar el cambio como nueva historia, no como modificación silenciosa.</t>
+        </is>
+      </c>
+      <c r="I12" s="50" t="n"/>
+      <c r="J12" s="50" t="n"/>
+      <c r="K12" s="50" t="n"/>
+      <c r="L12" s="50" t="n"/>
+      <c r="M12" s="50" t="n"/>
+      <c r="N12" s="50" t="n"/>
+      <c r="O12" s="50" t="n"/>
+      <c r="P12" s="50" t="n"/>
+      <c r="Q12" s="50" t="n"/>
+      <c r="R12" s="50" t="n"/>
+      <c r="S12" s="50" t="n"/>
+      <c r="T12" s="50" t="n"/>
+      <c r="U12" s="50" t="n"/>
+      <c r="V12" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="W12" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="X12" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="Y12" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z12" s="50" t="n"/>
+      <c r="AA12" s="50" t="n"/>
+      <c r="AB12" s="50" t="n"/>
+    </row>
+    <row r="13" ht="46" customHeight="1" s="32">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>El alcance crece más allá de lo escrito en las historias</t>
+        </is>
+      </c>
+      <c r="D13" s="49" t="inlineStr">
+        <is>
+          <t>Durante el desarrollo es común que aparezcan funcionalidades 'pequeñas' adicionales que parecen necesarias. Si no se controlan, suman trabajo no estimado y consumen sprints completos.</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F13" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G13" s="48" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="H13" s="49" t="inlineStr">
+        <is>
+          <t>Regla no negociable: no se programa nada que no esté en historia aprobada. Si surge una necesidad nueva, se documenta como historia adicional y se prioriza en sprint planning, no se agrega silenciosamente al sprint actual.</t>
+        </is>
+      </c>
+      <c r="I13" s="50" t="n"/>
+      <c r="J13" s="50" t="n"/>
+      <c r="K13" s="50" t="n"/>
+      <c r="L13" s="50" t="n"/>
+      <c r="M13" s="50" t="n"/>
+      <c r="N13" s="50" t="n"/>
+      <c r="O13" s="50" t="n"/>
+      <c r="P13" s="50" t="n"/>
+      <c r="Q13" s="50" t="n"/>
+      <c r="R13" s="50" t="n"/>
+      <c r="S13" s="50" t="n"/>
+      <c r="T13" s="50" t="n"/>
+      <c r="U13" s="50" t="n"/>
+      <c r="V13" s="51" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="W13" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X13" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Y13" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="Z13" s="50" t="n"/>
+      <c r="AA13" s="50" t="n"/>
+      <c r="AB13" s="50" t="n"/>
+    </row>
+    <row r="14" ht="46" customHeight="1" s="32">
+      <c r="A14" s="48" t="inlineStr">
+        <is>
+          <t>R-11</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>Mala interpretación de algún artículo LOPSRM/RLOPSRM en una historia</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="inlineStr">
+        <is>
+          <t>El equipo no son abogados. Es posible que la implementación de plazos (Art. 54), afirmativa ficta (Art. 133 RLOPSRM) o penalizaciones (Art. 46 Bis) tenga matices que no captamos correctamente y el cliente lo detecte en revisión.</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F14" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G14" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H14" s="49" t="inlineStr">
+        <is>
+          <t>Revisar el texto oficial publicado en el DOF antes de implementar reglas de negocio basadas en artículos legales. Documentar la interpretación adoptada en la historia correspondiente. Estar preparados para ajustar si el cliente señala una mala interpretación.</t>
+        </is>
+      </c>
+      <c r="I14" s="50" t="n"/>
+      <c r="J14" s="50" t="n"/>
+      <c r="K14" s="50" t="n"/>
+      <c r="L14" s="50" t="n"/>
+      <c r="M14" s="50" t="n"/>
+      <c r="N14" s="50" t="n"/>
+      <c r="O14" s="50" t="n"/>
+      <c r="P14" s="50" t="n"/>
+      <c r="Q14" s="50" t="n"/>
+      <c r="R14" s="50" t="n"/>
+      <c r="S14" s="50" t="n"/>
+      <c r="T14" s="50" t="n"/>
+      <c r="U14" s="50" t="n"/>
+      <c r="V14" s="50" t="n"/>
+      <c r="W14" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X14" s="53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="Y14" s="53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="Z14" s="50" t="n"/>
+      <c r="AA14" s="50" t="n"/>
+      <c r="AB14" s="50" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1" s="32">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>R-12</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Entrega</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>Maquetas no aprobadas a tiempo bloquean el sprint correspondiente</t>
+        </is>
+      </c>
+      <c r="D15" s="49" t="inlineStr">
+        <is>
+          <t>La regla no negociable es: maquetas aprobadas antes de programar. Si la aprobación de las maquetas se retrasa o se solicitan ajustes, el sprint puede arrancar tarde.</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F15" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="G15" s="48" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H15" s="49" t="inlineStr">
+        <is>
+          <t>Entregar maquetas con anticipación, no el mismo día que arranca el sprint. Tener maquetas de varios sprints listas para que si una no se aprueba, el equipo pueda avanzar con otra historia diferente.</t>
+        </is>
+      </c>
+      <c r="I15" s="50" t="n"/>
+      <c r="J15" s="50" t="n"/>
+      <c r="K15" s="50" t="n"/>
+      <c r="L15" s="50" t="n"/>
+      <c r="M15" s="50" t="n"/>
+      <c r="N15" s="50" t="n"/>
+      <c r="O15" s="50" t="n"/>
+      <c r="P15" s="50" t="n"/>
+      <c r="Q15" s="50" t="n"/>
+      <c r="R15" s="50" t="n"/>
+      <c r="S15" s="50" t="n"/>
+      <c r="T15" s="50" t="n"/>
+      <c r="U15" s="50" t="n"/>
+      <c r="V15" s="50" t="n"/>
+      <c r="W15" s="52" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="X15" s="53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="Y15" s="53" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="Z15" s="50" t="n"/>
+      <c r="AA15" s="50" t="n"/>
+      <c r="AB15" s="50" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="32" min="1" max="1"/>
+    <col width="13" customWidth="1" style="32" min="2" max="2"/>
+    <col width="14" customWidth="1" style="32" min="3" max="3"/>
+    <col width="13" customWidth="1" style="32" min="4" max="4"/>
+    <col width="11" customWidth="1" style="32" min="5" max="5"/>
+    <col width="12" customWidth="1" style="32" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="45" t="inlineStr">
+        <is>
+          <t>Resumen de evolución semanal de riesgos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="B3" s="47" t="inlineStr">
+        <is>
+          <t>Riesgos ALTA</t>
+        </is>
+      </c>
+      <c r="C3" s="47" t="inlineStr">
+        <is>
+          <t>Riesgos MEDIA</t>
+        </is>
+      </c>
+      <c r="D3" s="47" t="inlineStr">
+        <is>
+          <t>Riesgos BAJA</t>
+        </is>
+      </c>
+      <c r="E3" s="47" t="inlineStr">
+        <is>
+          <t>Con dato</t>
+        </is>
+      </c>
+      <c r="F3" s="47" t="inlineStr">
+        <is>
+          <t>Pendientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>S1 02/02–08/02</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>S2 09/02–15/02</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>S3 16/02–22/02</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t>S4 23/02–01/03</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>S5 02/03–08/03</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>S6 09/03–15/03</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="54" t="inlineStr">
+        <is>
+          <t>S7 16/03–22/03</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="54" t="inlineStr">
+        <is>
+          <t>S8 23/03–29/03</t>
+        </is>
+      </c>
+      <c r="B11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
+          <t>S9 30/03–05/04</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="54" t="inlineStr">
+        <is>
+          <t>S10 06/04–12/04</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="54" t="inlineStr">
+        <is>
+          <t>S11 13/04–19/04</t>
+        </is>
+      </c>
+      <c r="B14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>S12 20/04–26/04</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t>S13 27/04–03/05</t>
+        </is>
+      </c>
+      <c r="B16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="56" t="inlineStr">
+        <is>
+          <t>S14 04/05–10/05</t>
+        </is>
+      </c>
+      <c r="B17" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F17" s="57" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="56" t="inlineStr">
+        <is>
+          <t>S15 11/05–17/05</t>
+        </is>
+      </c>
+      <c r="B18" s="57" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="56" t="inlineStr">
+        <is>
+          <t>S16 18/05–24/05</t>
+        </is>
+      </c>
+      <c r="B19" s="57" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="56" t="inlineStr">
+        <is>
+          <t>S17 25/05–31/05</t>
+        </is>
+      </c>
+      <c r="B20" s="57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="D20" s="57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="57" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="54" t="inlineStr">
+        <is>
+          <t>S18 01/06–07/06</t>
+        </is>
+      </c>
+      <c r="B21" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="inlineStr">
+        <is>
+          <t>S19 08/06–14/06</t>
+        </is>
+      </c>
+      <c r="B22" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="54" t="inlineStr">
+        <is>
+          <t>S20 15/06–21/06</t>
+        </is>
+      </c>
+      <c r="B23" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="55" t="n">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2795,7 +4562,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="80.09999999999999" customHeight="1" s="32">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -4161,7 +5927,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="28" t="inlineStr">
         <is>

</xml_diff>